<commit_message>
update solution to Exercise 4.3
</commit_message>
<xml_diff>
--- a/exSol/Ex3/Ex3_3.xlsx
+++ b/exSol/Ex3/Ex3_3.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="26130"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="28526"/>
   <workbookPr autoCompressPictures="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://stummuac-my.sharepoint.com/personal/55061111_ad_mmu_ac_uk/Documents/Teaching/ODE6G6Z3017_2324/3_Exercise_solution/Ex3/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://stummuac-my.sharepoint.com/personal/55061111_ad_mmu_ac_uk/Documents/Teaching/ODE6G6Z3017_2526/0_Notes_Jupyter/exSol/Ex3/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="3" documentId="14_{66BE585E-C517-4ED2-AC5A-E6822CD1C850}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B1BAD1BC-4D96-452D-A7BE-3B0CBFA2DDF0}"/>
+  <xr:revisionPtr revIDLastSave="4" documentId="14_{66BE585E-C517-4ED2-AC5A-E6822CD1C850}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{52A2D20E-22AB-4E05-9222-27F91C2DB563}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17640" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Ex3_3" sheetId="8" r:id="rId1"/>
@@ -1544,7 +1544,7 @@
       <c r="J18" s="8"/>
       <c r="K18" s="10">
         <f>J19-J17</f>
-        <v>7.3448971757683612E-4</v>
+        <v>7.4973220274998642E-4</v>
       </c>
       <c r="N18" s="17"/>
     </row>
@@ -1573,7 +1573,7 @@
       <c r="I19" s="8"/>
       <c r="J19" s="10">
         <f>I20-I18</f>
-        <v>2.9725508313016569E-4</v>
+        <v>3.1249756830331599E-4</v>
       </c>
       <c r="K19" s="8"/>
     </row>
@@ -1590,7 +1590,7 @@
       <c r="H20" s="8"/>
       <c r="I20" s="10">
         <f>H21-H19</f>
-        <v>-2.098316139858003E-3</v>
+        <v>-2.0830736546848527E-3</v>
       </c>
       <c r="J20" s="8"/>
       <c r="K20" s="8"/>
@@ -1615,7 +1615,7 @@
       <c r="G21" s="11"/>
       <c r="H21" s="10">
         <f>G22-G20</f>
-        <v>2.0141526048612191E-2</v>
+        <v>2.0156768533785341E-2</v>
       </c>
       <c r="I21" s="8"/>
       <c r="J21" s="8"/>
@@ -1629,7 +1629,7 @@
       <c r="F22" s="8"/>
       <c r="G22" s="10">
         <f>F23-F21</f>
-        <v>-0.19138946835145931</v>
+        <v>-0.19137422586628616</v>
       </c>
       <c r="H22" s="11"/>
       <c r="I22" s="8"/>
@@ -1646,12 +1646,12 @@
         <v>0.5</v>
       </c>
       <c r="E23" s="10">
-        <f>E21+0.1*(F21+(1/2)*G20+(5/12)*H19+(9/24)*I18)</f>
-        <v>-0.81990245065992751</v>
+        <f>E21+0.1*(F21+(1/2)*G20+(5/12)*H19+(9/24)*I18+(251/720)*J17)</f>
+        <v>-0.81991769314510066</v>
       </c>
       <c r="F23" s="10">
         <f>-E23-2*D23</f>
-        <v>-0.18009754934007249</v>
+        <v>-0.18008230685489934</v>
       </c>
       <c r="G23" s="11"/>
       <c r="H23" s="8"/>

</xml_diff>